<commit_message>
Refresh executed Duka sales analysis
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/excel/duka_branch_summary.xlsx
+++ b/excel/duka_branch_summary.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/46d53ed39e5b26fd/Desktop/expense tracker/postgres-performance-lab/plp-da-a3-duka-sales-exploration/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_F10C14E60330C8C9CC4E88AFD1B1AC413FB14C2B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E9DF01FF-13B9-4E49-BB29-FEE742A48DAE}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="11_F10C14E60330C8C9CC4E883231F6B76F3FB14C2B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FD127DF9-A798-4439-8E0A-C029D6D67CB6}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3856,7 +3856,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="SEENOI HPF" refreshedDate="46311.762389930554" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="1000" xr:uid="{1A0C1606-77F1-42D1-B0F5-057CF5516232}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="SEENOI HPF" refreshedDate="46320.572729050924" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="1000" xr:uid="{898FD825-6701-4ACF-B657-3AB7C2258CCC}">
   <cacheSource type="worksheet">
     <worksheetSource ref="A1:N1001" sheet="Orders"/>
   </cacheSource>
@@ -19930,7 +19930,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{D21250D4-ABF1-4269-8071-C1FAFFF2D186}" name="RevenueByBranchChannel" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{926481D9-E00C-4585-97AE-687C5B7D865B}" name="RevenueByBranchChannel" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="A4:D14" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="14">
     <pivotField compact="0" outline="0" showAll="0"/>

</xml_diff>

<commit_message>
Save completed Duka assignment outputs
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/excel/duka_branch_summary.xlsx
+++ b/excel/duka_branch_summary.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/46d53ed39e5b26fd/Desktop/expense tracker/postgres-performance-lab/plp-da-a3-duka-sales-exploration/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_F10C14E60330C8C9CC4E883231F6B76F3FB14C2B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FD127DF9-A798-4439-8E0A-C029D6D67CB6}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="11_F10C14E60330C8C9CC4E88CF01318D5B3EB14C2B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CCA7725C-8228-4BE8-A219-05FDAD697114}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3856,7 +3856,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="SEENOI HPF" refreshedDate="46320.572729050924" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="1000" xr:uid="{898FD825-6701-4ACF-B657-3AB7C2258CCC}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="SEENOI HPF" refreshedDate="46320.995448263886" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="1000" xr:uid="{EB0ED1E7-A942-43E9-B06E-907C7C167F01}">
   <cacheSource type="worksheet">
     <worksheetSource ref="A1:N1001" sheet="Orders"/>
   </cacheSource>
@@ -19930,7 +19930,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{926481D9-E00C-4585-97AE-687C5B7D865B}" name="RevenueByBranchChannel" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{E7CEC156-080B-46A7-8002-D4B3C6176DE5}" name="RevenueByBranchChannel" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="A4:D14" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="14">
     <pivotField compact="0" outline="0" showAll="0"/>

</xml_diff>